<commit_message>
Actualizacion datos REM 2026-07-06 09:40 (orquestador)
</commit_message>
<xml_diff>
--- a/output/2024_estado_nutricional_por_SS.xlsx
+++ b/output/2024_estado_nutricional_por_SS.xlsx
@@ -310,16 +310,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -335,7 +327,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -343,30 +335,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -665,276 +639,276 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:89">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AH1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AI1" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AJ1" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AK1" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AL1" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AN1" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AO1" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AP1" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AQ1" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AR1" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AS1" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AT1" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AU1" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AV1" t="s">
         <v>46</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AW1" t="s">
         <v>47</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AX1" t="s">
         <v>48</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AY1" t="s">
         <v>49</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="AZ1" t="s">
         <v>50</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BA1" t="s">
         <v>51</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BB1" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BC1" t="s">
         <v>53</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BD1" t="s">
         <v>54</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BE1" t="s">
         <v>55</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BF1" t="s">
         <v>56</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BG1" t="s">
         <v>57</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BH1" t="s">
         <v>58</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BI1" t="s">
         <v>59</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BJ1" t="s">
         <v>60</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BK1" t="s">
         <v>61</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BL1" t="s">
         <v>62</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BM1" t="s">
         <v>63</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BN1" t="s">
         <v>64</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BO1" t="s">
         <v>65</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BP1" t="s">
         <v>66</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BQ1" t="s">
         <v>67</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BR1" t="s">
         <v>68</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BS1" t="s">
         <v>69</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BT1" t="s">
         <v>70</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BU1" t="s">
         <v>71</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BV1" t="s">
         <v>72</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BW1" t="s">
         <v>73</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BX1" t="s">
         <v>74</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BY1" t="s">
         <v>75</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="BZ1" t="s">
         <v>76</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CA1" t="s">
         <v>77</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CB1" t="s">
         <v>78</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="CC1" t="s">
         <v>79</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="CD1" t="s">
         <v>80</v>
       </c>
-      <c r="CE1" s="1" t="s">
+      <c r="CE1" t="s">
         <v>81</v>
       </c>
-      <c r="CF1" s="1" t="s">
+      <c r="CF1" t="s">
         <v>82</v>
       </c>
-      <c r="CG1" s="1" t="s">
+      <c r="CG1" t="s">
         <v>83</v>
       </c>
-      <c r="CH1" s="1" t="s">
+      <c r="CH1" t="s">
         <v>84</v>
       </c>
-      <c r="CI1" s="1" t="s">
+      <c r="CI1" t="s">
         <v>85</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="CJ1" t="s">
         <v>86</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="CK1" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:89">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -1185,7 +1159,7 @@
       </c>
     </row>
     <row r="3" spans="1:89">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -1436,7 +1410,7 @@
       </c>
     </row>
     <row r="4" spans="1:89">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -1687,7 +1661,7 @@
       </c>
     </row>
     <row r="5" spans="1:89">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="6" spans="1:89">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -2189,7 +2163,7 @@
       </c>
     </row>
     <row r="7" spans="1:89">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">
@@ -2450,84 +2424,84 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>45</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>46</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>57</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>67</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>68</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>78</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -2604,7 +2578,7 @@
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -2681,7 +2655,7 @@
       </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -2758,7 +2732,7 @@
       </c>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -2835,7 +2809,7 @@
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -2912,7 +2886,7 @@
       </c>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">
@@ -2999,84 +2973,84 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>36</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>47</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>48</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>58</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>59</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>69</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>70</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>80</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -3153,7 +3127,7 @@
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -3230,7 +3204,7 @@
       </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -3307,7 +3281,7 @@
       </c>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -3384,7 +3358,7 @@
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -3461,7 +3435,7 @@
       </c>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">
@@ -3548,84 +3522,84 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>38</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>39</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>49</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>61</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>71</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>72</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>82</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -3684,7 +3658,7 @@
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -3743,7 +3717,7 @@
       </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -3802,7 +3776,7 @@
       </c>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -3861,7 +3835,7 @@
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -3920,7 +3894,7 @@
       </c>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">
@@ -3989,84 +3963,84 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>40</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>62</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>63</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>74</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>84</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -4143,7 +4117,7 @@
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -4220,7 +4194,7 @@
       </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -4297,7 +4271,7 @@
       </c>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -4374,7 +4348,7 @@
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -4451,7 +4425,7 @@
       </c>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">
@@ -4538,84 +4512,84 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>43</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>64</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>65</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>75</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>76</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>86</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>89</v>
       </c>
       <c r="B2">
@@ -4692,7 +4666,7 @@
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>90</v>
       </c>
       <c r="B3">
@@ -4769,7 +4743,7 @@
       </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>91</v>
       </c>
       <c r="B4">
@@ -4846,7 +4820,7 @@
       </c>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>92</v>
       </c>
       <c r="B5">
@@ -4923,7 +4897,7 @@
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6">
@@ -5000,7 +4974,7 @@
       </c>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>94</v>
       </c>
       <c r="B7">

</xml_diff>